<commit_message>
Add MOSFET parameter table and RDS(on)-Tj dataset
</commit_message>
<xml_diff>
--- a/data/mosfet_parameters.xlsx
+++ b/data/mosfet_parameters.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\Power-MOSFET-Thermal-Reliability-Analysis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Power-MOSFET-Thermal-Reliability-Analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9637802-2D27-4271-8E78-732F7134D81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12285"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Parameter</t>
   </si>
@@ -47,9 +48,6 @@
     <t>Condition</t>
   </si>
   <si>
-    <t>Source Page</t>
-  </si>
-  <si>
     <t>Drain-Source Voltage</t>
   </si>
   <si>
@@ -108,12 +106,33 @@
   </si>
   <si>
     <t>µA</t>
+  </si>
+  <si>
+    <t>Maximum rating</t>
+  </si>
+  <si>
+    <t>VGS=10V, DC current, Tj=25°C</t>
+  </si>
+  <si>
+    <t>VDS=VGS, ID=270µA, Tj=25°C</t>
+  </si>
+  <si>
+    <t>VGS=10V, ID=100A, Tj=25°C</t>
+  </si>
+  <si>
+    <t>Operating temperature</t>
+  </si>
+  <si>
+    <t>Top-side</t>
+  </si>
+  <si>
+    <t>VDS=120V, VGS=0V, Tj=25°C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -170,7 +189,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -180,8 +199,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -462,24 +487,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="31.2" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -488,121 +513,155 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="46.8" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="3">
+        <v>120</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="62.4" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="3">
+        <v>300</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" ht="46.8" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" ht="46.8" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="27" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" ht="62.4" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="54" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="3">
+        <v>175</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="62.4" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="54" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="3">
+        <v>0.42</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="62.4" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="40.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="E8" s="3">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="3"/>
+      <c r="G8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>